<commit_message>
added reorder to video overlay apps. Completed data for Drafting app
</commit_message>
<xml_diff>
--- a/Drafting.xlsx
+++ b/Drafting.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sportnzgroup-my.sharepoint.com/personal/sam_bremer_hpsnz_org_nz/Documents/Desktop/Scripts/CNZ PTA Tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="8_{0AAFF668-2312-4652-B8D5-022CE08E49F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64289196-417B-4CE4-8B2E-FF24445B2CDF}"/>
+  <xr:revisionPtr revIDLastSave="247" documentId="8_{0AAFF668-2312-4652-B8D5-022CE08E49F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59E56F65-CA72-48CF-8128-5946469DC260}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{9C1A523A-0577-4DB6-8794-7B2D8C7AB7EB}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="3" xr2:uid="{9C1A523A-0577-4DB6-8794-7B2D8C7AB7EB}"/>
   </bookViews>
   <sheets>
     <sheet name="Nilai Q" sheetId="1" r:id="rId1"/>
-    <sheet name="Nilai R1" sheetId="2" r:id="rId2"/>
+    <sheet name="HongKong Q" sheetId="3" r:id="rId2"/>
+    <sheet name="HongKong R1" sheetId="4" r:id="rId3"/>
+    <sheet name="HongKong F" sheetId="6" r:id="rId4"/>
+    <sheet name="Nilai R1" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="13">
   <si>
     <t>Dan</t>
   </si>
@@ -76,6 +79,9 @@
   </si>
   <si>
     <t>Cadence</t>
+  </si>
+  <si>
+    <t>Keegan</t>
   </si>
 </sst>
 </file>
@@ -703,6 +709,736 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A8EBF5E-876F-48EA-B4EF-A9566528BD0A}">
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1">
+        <v>2</v>
+      </c>
+      <c r="C1">
+        <v>3</v>
+      </c>
+      <c r="D1">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2">
+        <v>538</v>
+      </c>
+      <c r="F2">
+        <v>393</v>
+      </c>
+      <c r="G2">
+        <v>355</v>
+      </c>
+      <c r="H2">
+        <v>305</v>
+      </c>
+      <c r="I2">
+        <v>55.82</v>
+      </c>
+      <c r="J2">
+        <v>73.38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>567</v>
+      </c>
+      <c r="F3">
+        <v>423</v>
+      </c>
+      <c r="G3">
+        <v>327</v>
+      </c>
+      <c r="H3">
+        <v>381</v>
+      </c>
+      <c r="I3">
+        <v>79.040000000000006</v>
+      </c>
+      <c r="J3">
+        <v>108.34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>649</v>
+      </c>
+      <c r="F4">
+        <v>429</v>
+      </c>
+      <c r="G4">
+        <v>424</v>
+      </c>
+      <c r="H4">
+        <v>433</v>
+      </c>
+      <c r="I4">
+        <v>112.94</v>
+      </c>
+      <c r="J4">
+        <v>143.28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>514</v>
+      </c>
+      <c r="F5">
+        <v>417</v>
+      </c>
+      <c r="G5">
+        <v>357</v>
+      </c>
+      <c r="H5">
+        <v>418</v>
+      </c>
+      <c r="I5">
+        <v>146.94</v>
+      </c>
+      <c r="J5">
+        <v>157.13999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6">
+        <v>567</v>
+      </c>
+      <c r="F6">
+        <v>408</v>
+      </c>
+      <c r="G6">
+        <v>359</v>
+      </c>
+      <c r="H6">
+        <v>327</v>
+      </c>
+      <c r="I6">
+        <v>161.56</v>
+      </c>
+      <c r="J6">
+        <v>178.98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>563</v>
+      </c>
+      <c r="F7">
+        <v>430</v>
+      </c>
+      <c r="G7">
+        <v>332</v>
+      </c>
+      <c r="H7">
+        <v>367</v>
+      </c>
+      <c r="I7">
+        <v>183.3</v>
+      </c>
+      <c r="J7">
+        <v>206.26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>647</v>
+      </c>
+      <c r="F8">
+        <v>427</v>
+      </c>
+      <c r="G8">
+        <v>433</v>
+      </c>
+      <c r="H8">
+        <v>427</v>
+      </c>
+      <c r="I8">
+        <v>210.72</v>
+      </c>
+      <c r="J8">
+        <v>241.18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{570E5417-3B7A-4445-891A-7ED124169949}">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1">
+        <v>2</v>
+      </c>
+      <c r="C1">
+        <v>3</v>
+      </c>
+      <c r="D1">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>637</v>
+      </c>
+      <c r="F2">
+        <v>470</v>
+      </c>
+      <c r="G2">
+        <v>366</v>
+      </c>
+      <c r="H2">
+        <v>430</v>
+      </c>
+      <c r="I2">
+        <v>61.58</v>
+      </c>
+      <c r="J2">
+        <v>84.76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>602</v>
+      </c>
+      <c r="F3">
+        <v>397</v>
+      </c>
+      <c r="G3">
+        <v>390</v>
+      </c>
+      <c r="H3">
+        <v>387</v>
+      </c>
+      <c r="I3">
+        <v>89.53</v>
+      </c>
+      <c r="J3">
+        <v>112.56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>524</v>
+      </c>
+      <c r="F4">
+        <v>448</v>
+      </c>
+      <c r="G4">
+        <v>397</v>
+      </c>
+      <c r="H4">
+        <v>406</v>
+      </c>
+      <c r="I4">
+        <v>117.4</v>
+      </c>
+      <c r="J4">
+        <v>150.52000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5">
+        <v>590</v>
+      </c>
+      <c r="F5">
+        <v>431</v>
+      </c>
+      <c r="G5">
+        <v>334</v>
+      </c>
+      <c r="I5">
+        <v>148.4</v>
+      </c>
+      <c r="J5">
+        <v>175.02</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>574</v>
+      </c>
+      <c r="F6">
+        <v>385</v>
+      </c>
+      <c r="G6">
+        <v>408</v>
+      </c>
+      <c r="I6">
+        <v>179.32</v>
+      </c>
+      <c r="J6">
+        <v>202.9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>456</v>
+      </c>
+      <c r="F7">
+        <v>398</v>
+      </c>
+      <c r="G7">
+        <v>363</v>
+      </c>
+      <c r="I7">
+        <v>207.25</v>
+      </c>
+      <c r="J7">
+        <v>245.84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D971315D-8544-4793-A2F6-2F36DCA34A65}">
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1">
+        <v>2</v>
+      </c>
+      <c r="C1">
+        <v>3</v>
+      </c>
+      <c r="D1">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>562</v>
+      </c>
+      <c r="F2">
+        <v>408</v>
+      </c>
+      <c r="G2">
+        <v>346</v>
+      </c>
+      <c r="H2">
+        <v>368</v>
+      </c>
+      <c r="I2">
+        <v>56.42</v>
+      </c>
+      <c r="J2">
+        <v>73.260000000000005</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>581</v>
+      </c>
+      <c r="F3">
+        <v>431</v>
+      </c>
+      <c r="G3">
+        <v>380</v>
+      </c>
+      <c r="H3">
+        <v>392</v>
+      </c>
+      <c r="I3">
+        <v>78.819999999999993</v>
+      </c>
+      <c r="J3">
+        <v>100.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>594</v>
+      </c>
+      <c r="F4">
+        <v>424</v>
+      </c>
+      <c r="G4">
+        <v>388</v>
+      </c>
+      <c r="H4">
+        <v>400</v>
+      </c>
+      <c r="I4">
+        <v>106.64</v>
+      </c>
+      <c r="J4">
+        <v>135.58000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>610</v>
+      </c>
+      <c r="F5">
+        <v>451</v>
+      </c>
+      <c r="G5">
+        <v>415</v>
+      </c>
+      <c r="H5">
+        <v>463</v>
+      </c>
+      <c r="I5">
+        <v>139.85</v>
+      </c>
+      <c r="J5">
+        <v>149.52000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>583</v>
+      </c>
+      <c r="F6">
+        <v>411</v>
+      </c>
+      <c r="G6">
+        <v>359</v>
+      </c>
+      <c r="I6">
+        <v>150.68</v>
+      </c>
+      <c r="J6">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>584</v>
+      </c>
+      <c r="F7">
+        <v>452</v>
+      </c>
+      <c r="G7">
+        <v>392</v>
+      </c>
+      <c r="I7">
+        <v>182.68</v>
+      </c>
+      <c r="J7">
+        <v>204.98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>651</v>
+      </c>
+      <c r="F8">
+        <v>497</v>
+      </c>
+      <c r="G8">
+        <v>462</v>
+      </c>
+      <c r="I8">
+        <v>209.14</v>
+      </c>
+      <c r="J8">
+        <v>230.02</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2F48074-F3A3-4879-89E6-1969009770B7}">
   <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>

</xml_diff>